<commit_message>
test(whitebox): synchronize assertions, expand branch coverage to 99.56% and update test docs
</commit_message>
<xml_diff>
--- a/docs/testing/DEF.xlsx
+++ b/docs/testing/DEF.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1631,6 +1631,288 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>DEF-BVA-ORD-001</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ORD</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Tạo món &amp; Tính tiền đơn hàng</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Tràn kiểu dữ liệu DECIMAL(10,2) trong CSDL PostgreSQL khi đơn giá lớn (100.000.000đ)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>TC_BVA_1.03, TC_BVA_1.04, TC_BVA_2.01, TC_BVA_2.03</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Khi tạo món với giá 100.000.000đ hoặc tính tổng tiền đơn hàng lớn, CSDL Supabase PostgreSQL báo lỗi "numeric field overflow" do cột chỉ định nghĩa DECIMAL(10,2). Đã fix bằng cách ALTER TABLE mở rộng sang DECIMAL(15,2) và giới hạn giá tối đa 100.000.000đ trong productController.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>DEF-BVA-RES-001</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>RES</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Đặt bàn &amp; Kiểm tra bàn trống</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Lỗi cú pháp DATE_ADD (MySQL) trên CSDL PostgreSQL Supabase khi tạo đặt bàn</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>BVA-RES-01, BVA-RES-02, BVA-RES-03, BVA-RES-04, BVA-RES-05, BVA-RES-06, BVA-RES-07, BVA-RES-08, BVA-RES-09, BVA-RES-10</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Hàm createReservation sử dụng hàm DATE_ADD(reservationTime, INTERVAL 2 HOUR) của MySQL khiến PostgreSQL báo lỗi syntax error "2" và trả về HTTP 500. Đã fix bằng cách thay thế sang khoảng thời gian Date trong JavaScript ([Op.gt]: overlapStartWindow, [Op.lt]: endTime) tương thích chuẩn mọi CSDL.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DEF-BVA-RES-002</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>RES</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Nhận bàn (Check-in)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Độ trễ mạng gây lệch thời gian biên check-in 30 phút dẫn đến bị từ chối 400</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>BVA-RES-01</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Khi check-in tại mốc biên đúng 30 phút, độ trễ mạng HTTP round-trip (khoảng 1s) làm diffMins = 30.02 &gt; 30 khiến request bị từ chối với HTTP 400. Đã fix bằng cách áp dụng Math.round(diffMins) để bù trừ độ trễ mạng hợp lý.</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>DEF-EP-PNT-001</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>PNT</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Tích điểm khách hàng</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Số điện thoại sai định dạng chứa chữ không bị chặn validate mà trả về HTTP 404</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>TC_EP_07, EP-POINT-007</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Khi gửi số điện thoại sai định dạng (vd: 09012abcde), API không validate regex mà query CSDL và trả về HTTP 404 Not Found thay vì HTTP 400 Bad Request. Đã fix bằng cách bổ sung Regex kiểm tra định dạng SĐT Việt Nam (/^(0|\+84)[0-9]{9,10}$/) trong pointController.js.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>DEF-BVA-PNT-001</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>PNT</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Tích điểm trần</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Điểm tích lũy vượt mức tối đa 10.000.000 điểm không được chặn làm tròn trần</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>BVA-POINT-004, BVA-POINT-005</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Khi tổng điểm tích lũy của khách hàng cộng thêm điểm mới vượt quá 10.000.000 điểm, hệ thống cần chặn không cho vượt trần MAX_POINTS. Đã bổ sung Math.min(MAX_POINTS, previousPoints + earnedPoints) trong pointController.js.</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>DEF-BVA-TAB-001</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Quản lý bàn ăn</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Thiếu validation số nguyên và khoảng giá trị cho tableNumber và capacity</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>BT-012-TB-001, BT-012-TB-002, BT-012-TB-003, BT-012-TB-004, BT-012-TB-005, BT-012-TB-006</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>API tạo bàn cho phép tableNumber/capacity là số thập phân, capacity &lt; 1 hoặc qrCode rỗng, status sai enum. Đã fix bằng cách bổ sung kiểm tra Number.isInteger, capacity &gt;= 1, validate qrCode và enum AVAILABLE/OCCUPIED trong tableController.js.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>